<commit_message>
have good random positioning now
</commit_message>
<xml_diff>
--- a/Timings.xlsx
+++ b/Timings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEV\TESTS\gs\avis-gaussian-splatting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD597B57-E41B-4866-B8E4-70401EEEB69D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC5263D-1852-4E04-B4C2-5A4C99A2767B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5970" yWindow="1935" windowWidth="30795" windowHeight="15975" xr2:uid="{91218539-CA6E-4D46-9F47-0C4D7F2F2CA5}"/>
+    <workbookView xWindow="2610" yWindow="1470" windowWidth="22395" windowHeight="18285" xr2:uid="{91218539-CA6E-4D46-9F47-0C4D7F2F2CA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>16.06.</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
   <si>
     <t>Nr Of Points</t>
   </si>
@@ -50,22 +44,64 @@
     <t>Training Duration</t>
   </si>
   <si>
-    <t>PSNR</t>
-  </si>
-  <si>
-    <t>Method</t>
-  </si>
-  <si>
-    <t>Smart Initialization (DICOM-Colors)</t>
-  </si>
-  <si>
     <t>Resolution</t>
   </si>
   <si>
     <t>half</t>
   </si>
   <si>
-    <t>Loss</t>
+    <t>Smart Initialization</t>
+  </si>
+  <si>
+    <t>Random Initialization</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>17.06.</t>
+  </si>
+  <si>
+    <t>PSNR (Start)</t>
+  </si>
+  <si>
+    <t>Loss (Start)</t>
+  </si>
+  <si>
+    <t>Loss (End)</t>
+  </si>
+  <si>
+    <t>PSNR (End)</t>
+  </si>
+  <si>
+    <t>With Orientation, DICOM Colors</t>
+  </si>
+  <si>
+    <t>Without orientation, DICOM colors</t>
+  </si>
+  <si>
+    <t>WO Orientation, random Colors</t>
+  </si>
+  <si>
+    <t>W Orientation, random Colors</t>
+  </si>
+  <si>
+    <t>Bad Placement</t>
+  </si>
+  <si>
+    <t>Better Placement</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>b3594496-d</t>
+  </si>
+  <si>
+    <t>bb28143d-9</t>
+  </si>
+  <si>
+    <t>35445b03-3</t>
   </si>
 </sst>
 </file>
@@ -73,9 +109,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,16 +119,39 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -100,20 +159,53 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4"/>
+      </right>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4"/>
+      </right>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="25" formatCode="hh:mm"/>
     </dxf>
@@ -131,16 +223,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B23995EE-D1AC-4E6A-A91A-80AB79A654FE}" name="Tabelle1" displayName="Tabelle1" ref="C7:I21" totalsRowShown="0">
-  <autoFilter ref="C7:I21" xr:uid="{B23995EE-D1AC-4E6A-A91A-80AB79A654FE}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EA3F6830-BAC4-4FD9-A394-9E999F8033CE}" name="Date"/>
-    <tableColumn id="2" xr3:uid="{F091966C-55EF-48D3-B415-C56E9FE9AAC5}" name="Method"/>
-    <tableColumn id="3" xr3:uid="{4C1CFC3C-F530-4FFA-A8CA-ADF991176FFD}" name="Training Duration" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{E9B572CD-3E9A-4CEA-9B7C-305488712FFB}" name="Nr Of Points"/>
-    <tableColumn id="5" xr3:uid="{F7B34D60-0824-4BD2-B654-A34383077C04}" name="PSNR"/>
-    <tableColumn id="6" xr3:uid="{94FB43B6-19FB-4A94-A78E-1026CB6E37F2}" name="Resolution"/>
-    <tableColumn id="7" xr3:uid="{3B9F1CBC-2959-4830-89AB-95327E9D0F3B}" name="Loss"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B23995EE-D1AC-4E6A-A91A-80AB79A654FE}" name="Tabelle1" displayName="Tabelle1" ref="C7:J21" totalsRowShown="0">
+  <autoFilter ref="C7:J21" xr:uid="{B23995EE-D1AC-4E6A-A91A-80AB79A654FE}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{EA3F6830-BAC4-4FD9-A394-9E999F8033CE}" name="Code"/>
+    <tableColumn id="2" xr3:uid="{F091966C-55EF-48D3-B415-C56E9FE9AAC5}" name="Training Duration"/>
+    <tableColumn id="3" xr3:uid="{4C1CFC3C-F530-4FFA-A8CA-ADF991176FFD}" name="Nr Of Points" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{E9B572CD-3E9A-4CEA-9B7C-305488712FFB}" name="Resolution"/>
+    <tableColumn id="6" xr3:uid="{94FB43B6-19FB-4A94-A78E-1026CB6E37F2}" name="PSNR (Start)"/>
+    <tableColumn id="7" xr3:uid="{18CF464E-7E9E-4DB2-BCF0-CFB02527AC18}" name="PSNR (End)"/>
+    <tableColumn id="8" xr3:uid="{FDB7CFA4-5E00-479A-ADF7-E103BC1ED88C}" name="Loss (Start)"/>
+    <tableColumn id="9" xr3:uid="{B4B56141-5A8A-475C-ADE3-FD142F451865}" name="Loss (End)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{41A20CA5-4675-49BB-8958-E2F68EA96ED0}" name="Tabelle13" displayName="Tabelle13" ref="C26:K40" totalsRowShown="0">
+  <autoFilter ref="C26:K40" xr:uid="{41A20CA5-4675-49BB-8958-E2F68EA96ED0}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{5ADD7675-23D6-40D9-8031-52023CB23480}" name="Code"/>
+    <tableColumn id="2" xr3:uid="{14203E69-6608-483D-BBEB-EB038E259A23}" name="Training Duration"/>
+    <tableColumn id="3" xr3:uid="{5FE5403A-FE12-41A1-BE7D-0FC20267D7C4}" name="Nr Of Points" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{6BB98B40-3C2F-4659-B95E-6F199432AF52}" name="Resolution"/>
+    <tableColumn id="5" xr3:uid="{B4B69CDA-51CC-4214-89F5-CD30E8EB4931}" name="PSNR (Start)"/>
+    <tableColumn id="6" xr3:uid="{C2AAF3AF-1964-4907-9B53-4AAEF160B32B}" name="PSNR (End)"/>
+    <tableColumn id="7" xr3:uid="{33CAF3C7-8F0F-42A6-A2D8-A3625FCD81F9}" name="Loss (Start)"/>
+    <tableColumn id="8" xr3:uid="{5A2CABB3-9FD4-4659-A472-928036ED601F}" name="Loss (End)"/>
+    <tableColumn id="9" xr3:uid="{845B5EE9-5F9F-4A7C-AF02-F0D943496E19}" name="Comments"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -463,104 +574,340 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C03B34-FF9A-4BAB-BFFD-D449B574B7AC}">
-  <dimension ref="C7:I21"/>
+  <dimension ref="C5:K40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="34.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" customWidth="1"/>
     <col min="6" max="6" width="13.85546875" customWidth="1"/>
     <col min="8" max="8" width="12.5703125" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="12" max="12" width="14.85546875" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" customWidth="1"/>
+    <col min="15" max="15" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="3:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
         <v>0</v>
-      </c>
-      <c r="D7" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" t="s">
-        <v>3</v>
       </c>
       <c r="F7" t="s">
         <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H7" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="I7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>10</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.23958333333333334</v>
+      </c>
+      <c r="E8">
+        <v>100000</v>
+      </c>
+      <c r="F8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="4">
+        <v>26.5</v>
+      </c>
+      <c r="H8">
+        <v>30.5</v>
+      </c>
+      <c r="I8">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="J8">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.23611111111111113</v>
+      </c>
+      <c r="E9">
+        <v>100000</v>
+      </c>
+      <c r="F9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G9">
+        <v>26.65</v>
+      </c>
+      <c r="H9">
+        <v>30.7</v>
+      </c>
+      <c r="I9">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="J9">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0.21319444444444444</v>
+      </c>
+      <c r="E10">
+        <v>100000</v>
+      </c>
+      <c r="F10" t="s">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>30.29</v>
+      </c>
+      <c r="H10">
+        <v>34.6</v>
+      </c>
+      <c r="I10">
+        <v>1.2E-2</v>
+      </c>
+      <c r="J10">
+        <v>7.9000000000000008E-3</v>
+      </c>
+      <c r="K10" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.21319444444444444</v>
+      </c>
+      <c r="E11">
+        <v>100000</v>
+      </c>
+      <c r="F11" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11">
+        <v>30.35</v>
+      </c>
+      <c r="H11">
+        <v>35.1</v>
+      </c>
+      <c r="I11">
+        <v>1.2E-2</v>
+      </c>
+      <c r="J11">
+        <v>7.7000000000000002E-3</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="K12" s="8"/>
+    </row>
+    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="K13" s="8"/>
+    </row>
+    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="K14" s="8"/>
+    </row>
+    <row r="15" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E15" s="1"/>
+      <c r="K15" s="8"/>
+    </row>
+    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E16" s="1"/>
+      <c r="K16" s="8"/>
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E17" s="1"/>
+      <c r="K17" s="8"/>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E18" s="1"/>
+      <c r="K18" s="8"/>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E19" s="1"/>
+      <c r="K19" s="8"/>
+    </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E20" s="1"/>
+      <c r="K20" s="8"/>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E21" s="1"/>
+      <c r="K21" s="9"/>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" t="s">
         <v>1</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E26" t="s">
+        <v>0</v>
+      </c>
+      <c r="F26" t="s">
+        <v>2</v>
+      </c>
+      <c r="G26" t="s">
+        <v>8</v>
+      </c>
+      <c r="H26" t="s">
+        <v>11</v>
+      </c>
+      <c r="I26" t="s">
+        <v>9</v>
+      </c>
+      <c r="J26" t="s">
+        <v>10</v>
+      </c>
+      <c r="K26" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="3">
-        <v>3.8194444444444443E-3</v>
-      </c>
-      <c r="F8">
+    </row>
+    <row r="27" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0.19999999999999998</v>
+      </c>
+      <c r="E27" s="4">
         <v>100000</v>
       </c>
-      <c r="G8">
-        <v>32.65</v>
-      </c>
-      <c r="H8" t="s">
-        <v>8</v>
-      </c>
-      <c r="I8">
-        <v>9.9500000000000005E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="E16" s="1"/>
-    </row>
-    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E18" s="1"/>
-    </row>
-    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E21" s="1"/>
+      <c r="F27" t="s">
+        <v>3</v>
+      </c>
+      <c r="G27">
+        <v>26.81</v>
+      </c>
+      <c r="H27">
+        <v>30.76</v>
+      </c>
+      <c r="I27">
+        <v>1.9E-2</v>
+      </c>
+      <c r="J27">
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="K27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="1">
+        <v>0.26319444444444445</v>
+      </c>
+      <c r="E28" s="4">
+        <v>100000</v>
+      </c>
+      <c r="F28" t="s">
+        <v>3</v>
+      </c>
+      <c r="G28">
+        <v>25.88</v>
+      </c>
+      <c r="H28">
+        <v>30.01</v>
+      </c>
+      <c r="I28">
+        <v>1.47E-2</v>
+      </c>
+      <c r="J28">
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="K28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E31" s="1"/>
+    </row>
+    <row r="32" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="E32" s="1"/>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="1"/>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="1"/>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E35" s="1"/>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="1"/>
+    </row>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="1"/>
+    </row>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E38" s="1"/>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E39" s="1"/>
+    </row>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E40" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>